<commit_message>
update the xl file and adde instructions not to pull in bad links
</commit_message>
<xml_diff>
--- a/uploaded_files/EMERGE Content - Capstone ITSMF.xlsx
+++ b/uploaded_files/EMERGE Content - Capstone ITSMF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aieshadotson/Code_Repos/ITSMF_Chatbot/chatbot-prototype/uploaded_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA309CD-B307-4744-96C1-2D377B5BC914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC512398-5FD4-8042-8A97-21332BDE1915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="1040" windowWidth="60160" windowHeight="28240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1040" windowWidth="60160" windowHeight="28240" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legend" sheetId="1" r:id="rId1"/>
@@ -98,9 +98,6 @@
     <t xml:space="preserve">FAQ, General Inquiry         </t>
   </si>
   <si>
-    <t>Emerge Academy, women</t>
-  </si>
-  <si>
     <t>Q2</t>
   </si>
   <si>
@@ -108,9 +105,6 @@
   </si>
   <si>
     <t>ITSMF Management Academy fuels the initiative of mid-level professionals by connecting them to resources that fully develop their management skills and emotional intelligence. Participants forge enduring relationships with their peers who understand their challenges, and advance through unfettered access to industry-leading executives whose experiences and instruction are instrumental in guiding their personal and professional growth. Graduates are focused, visionary leaders and architects of positive organizational change.</t>
-  </si>
-  <si>
-    <t>Management Academy, Mid-Level professional</t>
   </si>
   <si>
     <t>Q3</t>
@@ -2081,6 +2075,12 @@
   <si>
     <t xml:space="preserve">ITSMF increases the representation of professionals at senior levels in technology, to impact organizational innovation and growth. We do this by developing and nurturing these dynamic leaders through enrichment of the mind, body and soul.
 </t>
+  </si>
+  <si>
+    <t>Emerge Academy, women, women only</t>
+  </si>
+  <si>
+    <t>Management Academy, Mid-Level professional, men, women</t>
   </si>
 </sst>
 </file>
@@ -4755,7 +4755,7 @@
         <v>22</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>23</v>
+        <v>415</v>
       </c>
       <c r="F2" s="17">
         <v>45718</v>
@@ -4765,19 +4765,19 @@
     </row>
     <row r="3" spans="1:8" ht="91">
       <c r="A3" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="C3" s="15" t="s">
         <v>25</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>26</v>
       </c>
       <c r="D3" s="22" t="s">
         <v>22</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>27</v>
+        <v>416</v>
       </c>
       <c r="F3" s="23">
         <v>45718</v>
@@ -4787,19 +4787,19 @@
     </row>
     <row r="4" spans="1:8" ht="98">
       <c r="A4" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>28</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>30</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F4" s="17">
         <v>45718</v>
@@ -4809,19 +4809,19 @@
     </row>
     <row r="5" spans="1:8" ht="70">
       <c r="A5" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="21" t="s">
         <v>32</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>34</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>22</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F5" s="23">
         <v>45718</v>
@@ -4831,19 +4831,19 @@
     </row>
     <row r="6" spans="1:8" ht="91">
       <c r="A6" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>36</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>38</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F6" s="17">
         <v>45718</v>
@@ -4853,19 +4853,19 @@
     </row>
     <row r="7" spans="1:8" ht="143">
       <c r="A7" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>40</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>42</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F7" s="23">
         <v>45718</v>
@@ -4875,19 +4875,19 @@
     </row>
     <row r="8" spans="1:8" ht="117">
       <c r="A8" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="26" t="s">
         <v>44</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>46</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F8" s="17">
         <v>45718</v>
@@ -4897,19 +4897,19 @@
     </row>
     <row r="9" spans="1:8" ht="169">
       <c r="A9" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="26" t="s">
         <v>48</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>50</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F9" s="23">
         <v>45718</v>
@@ -4919,19 +4919,19 @@
     </row>
     <row r="10" spans="1:8" ht="28">
       <c r="A10" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="26" t="s">
         <v>52</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>54</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>22</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F10" s="17">
         <v>45718</v>
@@ -4941,19 +4941,19 @@
     </row>
     <row r="11" spans="1:8" ht="28">
       <c r="A11" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="26" t="s">
         <v>56</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>58</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>22</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F11" s="23">
         <v>45718</v>
@@ -4963,19 +4963,19 @@
     </row>
     <row r="12" spans="1:8" ht="28">
       <c r="A12" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="16" t="s">
         <v>60</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>62</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F12" s="17">
         <v>45718</v>
@@ -4985,19 +4985,19 @@
     </row>
     <row r="13" spans="1:8" ht="28">
       <c r="A13" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="26" t="s">
         <v>64</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>66</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F13" s="23">
         <v>45718</v>
@@ -5007,19 +5007,19 @@
     </row>
     <row r="14" spans="1:8" ht="52">
       <c r="A14" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="27" t="s">
         <v>67</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>69</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F14" s="17">
         <v>45718</v>
@@ -5029,19 +5029,19 @@
     </row>
     <row r="15" spans="1:8" ht="42">
       <c r="A15" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>71</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>73</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>22</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F15" s="23">
         <v>45718</v>
@@ -5051,19 +5051,19 @@
     </row>
     <row r="16" spans="1:8" ht="28">
       <c r="A16" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="28" t="s">
         <v>75</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>77</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>22</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F16" s="17">
         <v>45718</v>
@@ -5073,19 +5073,19 @@
     </row>
     <row r="17" spans="1:8" ht="42">
       <c r="A17" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="26" t="s">
         <v>79</v>
-      </c>
-      <c r="B17" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" s="26" t="s">
-        <v>81</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>22</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F17" s="23">
         <v>45718</v>
@@ -5095,19 +5095,19 @@
     </row>
     <row r="18" spans="1:8" ht="45.75" customHeight="1">
       <c r="A18" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="D18" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="E18" s="14" t="s">
         <v>85</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>87</v>
       </c>
       <c r="F18" s="17">
         <v>45718</v>
@@ -5117,19 +5117,19 @@
     </row>
     <row r="19" spans="1:8" ht="42">
       <c r="A19" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E19" s="21" t="s">
         <v>88</v>
-      </c>
-      <c r="B19" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>90</v>
       </c>
       <c r="F19" s="23">
         <v>45718</v>
@@ -5139,19 +5139,19 @@
     </row>
     <row r="20" spans="1:8" ht="28">
       <c r="A20" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="D20" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="14" t="s">
         <v>92</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>94</v>
       </c>
       <c r="F20" s="17">
         <v>45718</v>
@@ -5161,19 +5161,19 @@
     </row>
     <row r="21" spans="1:8" ht="42">
       <c r="A21" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="D21" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E21" s="21" t="s">
         <v>96</v>
-      </c>
-      <c r="C21" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="E21" s="21" t="s">
-        <v>98</v>
       </c>
       <c r="F21" s="23">
         <v>45718</v>
@@ -5183,19 +5183,19 @@
     </row>
     <row r="22" spans="1:8" ht="28">
       <c r="A22" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="D22" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="14" t="s">
         <v>100</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>102</v>
       </c>
       <c r="F22" s="17">
         <v>45718</v>
@@ -5205,19 +5205,19 @@
     </row>
     <row r="23" spans="1:8" ht="28">
       <c r="A23" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="C23" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>105</v>
-      </c>
       <c r="D23" s="21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F23" s="23">
         <v>45718</v>
@@ -5227,19 +5227,19 @@
     </row>
     <row r="24" spans="1:8" ht="28">
       <c r="A24" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>108</v>
-      </c>
       <c r="D24" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F24" s="17">
         <v>45718</v>
@@ -5249,19 +5249,19 @@
     </row>
     <row r="25" spans="1:8" ht="28">
       <c r="A25" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="B25" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="C25" s="26" t="s">
-        <v>111</v>
-      </c>
       <c r="D25" s="21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E25" s="21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F25" s="23">
         <v>45718</v>
@@ -5271,19 +5271,19 @@
     </row>
     <row r="26" spans="1:8" ht="28">
       <c r="A26" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="D26" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26" s="14" t="s">
         <v>113</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="D26" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>115</v>
       </c>
       <c r="F26" s="17">
         <v>45718</v>
@@ -5293,19 +5293,19 @@
     </row>
     <row r="27" spans="1:8" ht="28">
       <c r="A27" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="C27" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="C27" s="30" t="s">
-        <v>118</v>
-      </c>
       <c r="D27" s="21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E27" s="21" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F27" s="23">
         <v>45718</v>
@@ -5313,19 +5313,19 @@
     </row>
     <row r="28" spans="1:8" ht="28">
       <c r="A28" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C28" s="31" t="s">
         <v>119</v>
       </c>
-      <c r="B28" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C28" s="31" t="s">
-        <v>121</v>
-      </c>
       <c r="D28" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F28" s="17">
         <v>45718</v>
@@ -5335,19 +5335,19 @@
     </row>
     <row r="29" spans="1:8" ht="28">
       <c r="A29" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="C29" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="B29" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="C29" s="32" t="s">
-        <v>124</v>
-      </c>
       <c r="D29" s="21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F29" s="23">
         <v>45718</v>
@@ -5648,16 +5648,16 @@
         <v>19</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="E2" s="14" t="s">
         <v>126</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>128</v>
       </c>
       <c r="F2" s="43">
         <v>45719</v>
@@ -5669,19 +5669,19 @@
     </row>
     <row r="3" spans="1:8" ht="84">
       <c r="A3" s="45" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F3" s="46">
         <v>45719</v>
@@ -5693,19 +5693,19 @@
     </row>
     <row r="4" spans="1:8" ht="98">
       <c r="A4" s="42" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>131</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>133</v>
       </c>
       <c r="F4" s="43">
         <v>45719</v>
@@ -5717,19 +5717,19 @@
     </row>
     <row r="5" spans="1:8" ht="14">
       <c r="A5" s="45" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="21" t="s">
         <v>134</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>136</v>
       </c>
       <c r="F5" s="46">
         <v>45719</v>
@@ -5741,19 +5741,19 @@
     </row>
     <row r="6" spans="1:8" ht="14">
       <c r="A6" s="42" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>137</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>139</v>
       </c>
       <c r="F6" s="43">
         <v>45719</v>
@@ -5765,19 +5765,19 @@
     </row>
     <row r="7" spans="1:8" ht="28">
       <c r="A7" s="45" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="21" t="s">
+        <v>138</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="21" t="s">
         <v>140</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>141</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>142</v>
       </c>
       <c r="F7" s="46">
         <v>45719</v>
@@ -5789,19 +5789,19 @@
     </row>
     <row r="8" spans="1:8" ht="14">
       <c r="A8" s="42" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>145</v>
       </c>
       <c r="F8" s="43">
         <v>45719</v>
@@ -5813,19 +5813,19 @@
     </row>
     <row r="9" spans="1:8" ht="14">
       <c r="A9" s="45" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="E9" s="21" t="s">
         <v>146</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>148</v>
       </c>
       <c r="F9" s="46">
         <v>45719</v>
@@ -5837,19 +5837,19 @@
     </row>
     <row r="10" spans="1:8" ht="224">
       <c r="A10" s="42" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>149</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>151</v>
       </c>
       <c r="F10" s="43">
         <v>45719</v>
@@ -5861,19 +5861,19 @@
     </row>
     <row r="11" spans="1:8" ht="28">
       <c r="A11" s="45" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F11" s="46">
         <v>45719</v>
@@ -5885,19 +5885,19 @@
     </row>
     <row r="12" spans="1:8" ht="168">
       <c r="A12" s="42" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F12" s="43">
         <v>45719</v>
@@ -5909,19 +5909,19 @@
     </row>
     <row r="13" spans="1:8" ht="56">
       <c r="A13" s="45" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F13" s="46">
         <v>45719</v>
@@ -5933,19 +5933,19 @@
     </row>
     <row r="14" spans="1:8" ht="154">
       <c r="A14" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="D14" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E14" s="14" t="s">
         <v>159</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>161</v>
       </c>
       <c r="F14" s="43">
         <v>45719</v>
@@ -5957,19 +5957,19 @@
     </row>
     <row r="15" spans="1:8" ht="140">
       <c r="A15" s="45" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B15" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>397</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>159</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>399</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>161</v>
       </c>
       <c r="F15" s="46">
         <v>45719</v>
@@ -5981,19 +5981,19 @@
     </row>
     <row r="16" spans="1:8" ht="154">
       <c r="A16" s="42" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E16" s="14" t="s">
         <v>159</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>161</v>
       </c>
       <c r="F16" s="43">
         <v>45719</v>
@@ -6005,19 +6005,19 @@
     </row>
     <row r="17" spans="1:8" ht="42">
       <c r="A17" s="45" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B17" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>164</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="E17" s="21" t="s">
         <v>159</v>
-      </c>
-      <c r="C17" s="34" t="s">
-        <v>166</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>161</v>
       </c>
       <c r="F17" s="46">
         <v>45720</v>
@@ -6029,19 +6029,19 @@
     </row>
     <row r="18" spans="1:8" ht="196">
       <c r="A18" s="42" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B18" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" s="14" t="s">
         <v>167</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>169</v>
       </c>
       <c r="F18" s="43"/>
       <c r="G18" s="43"/>
@@ -14973,16 +14973,16 @@
         <v>19</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="D2" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="E2" s="18" t="s">
         <v>171</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>172</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>173</v>
       </c>
       <c r="F2" s="17">
         <v>45716</v>
@@ -14991,24 +14991,24 @@
         <v>45718</v>
       </c>
       <c r="H2" s="129" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="117">
       <c r="A3" s="58" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" s="126" t="s">
+        <v>399</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="E3" s="24" t="s">
         <v>174</v>
-      </c>
-      <c r="C3" s="126" t="s">
-        <v>401</v>
-      </c>
-      <c r="D3" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>176</v>
       </c>
       <c r="F3" s="23">
         <v>45716</v>
@@ -15017,24 +15017,24 @@
         <v>45718</v>
       </c>
       <c r="H3" s="130" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="14">
       <c r="A4" s="57" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="E4" s="18" t="s">
         <v>179</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>180</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>181</v>
       </c>
       <c r="F4" s="17">
         <v>45716</v>
@@ -15046,19 +15046,19 @@
     </row>
     <row r="5" spans="1:8" ht="14">
       <c r="A5" s="58" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" s="24" t="s">
+        <v>180</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="E5" s="24" t="s">
         <v>182</v>
-      </c>
-      <c r="C5" s="59" t="s">
-        <v>183</v>
-      </c>
-      <c r="D5" s="24" t="s">
-        <v>180</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>184</v>
       </c>
       <c r="F5" s="23">
         <v>45716</v>
@@ -15070,19 +15070,19 @@
     </row>
     <row r="6" spans="1:8" ht="14">
       <c r="A6" s="57" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="E6" s="18" t="s">
         <v>185</v>
-      </c>
-      <c r="C6" s="59" t="s">
-        <v>186</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>180</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>187</v>
       </c>
       <c r="F6" s="17">
         <v>45716</v>
@@ -15094,19 +15094,19 @@
     </row>
     <row r="7" spans="1:8" ht="14">
       <c r="A7" s="58" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="E7" s="24" t="s">
         <v>189</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>191</v>
       </c>
       <c r="F7" s="23">
         <v>45716</v>
@@ -15118,19 +15118,19 @@
     </row>
     <row r="8" spans="1:8" ht="143">
       <c r="A8" s="57" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F8" s="17">
         <v>45716</v>
@@ -15139,24 +15139,24 @@
         <v>45718</v>
       </c>
       <c r="H8" s="133" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="14">
       <c r="A9" s="58" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>400</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="E9" s="24" t="s">
         <v>194</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>402</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>195</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>196</v>
       </c>
       <c r="F9" s="23">
         <v>45716</v>
@@ -15168,19 +15168,19 @@
     </row>
     <row r="10" spans="1:8" ht="14">
       <c r="A10" s="57" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="E10" s="18" t="s">
         <v>198</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>200</v>
       </c>
       <c r="F10" s="17">
         <v>45716</v>
@@ -15192,19 +15192,19 @@
     </row>
     <row r="11" spans="1:8" ht="14">
       <c r="A11" s="58" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B11" s="60" t="s">
+        <v>199</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="D11" s="24" t="s">
         <v>201</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="E11" s="24" t="s">
         <v>202</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="E11" s="24" t="s">
-        <v>204</v>
       </c>
       <c r="F11" s="23">
         <v>45716</v>
@@ -15213,24 +15213,24 @@
         <v>45718</v>
       </c>
       <c r="H11" s="128" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="13">
       <c r="A12" s="57" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="C12" s="61" t="s">
+        <v>205</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="C12" s="61" t="s">
+      <c r="E12" s="18" t="s">
         <v>207</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>208</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>209</v>
       </c>
       <c r="F12" s="17">
         <v>45716</v>
@@ -15242,19 +15242,19 @@
     </row>
     <row r="13" spans="1:8" ht="28">
       <c r="A13" s="58" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" s="24" t="s">
+        <v>208</v>
+      </c>
+      <c r="C13" s="127" t="s">
+        <v>401</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="E13" s="24" t="s">
         <v>210</v>
-      </c>
-      <c r="C13" s="127" t="s">
-        <v>403</v>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>211</v>
-      </c>
-      <c r="E13" s="24" t="s">
-        <v>212</v>
       </c>
       <c r="F13" s="23">
         <v>45716</v>
@@ -15263,24 +15263,24 @@
         <v>45718</v>
       </c>
       <c r="H13" s="130" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="13">
       <c r="A14" s="57" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="C14" s="61" t="s">
+        <v>212</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="E14" s="18" t="s">
         <v>213</v>
-      </c>
-      <c r="C14" s="61" t="s">
-        <v>214</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>203</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>215</v>
       </c>
       <c r="F14" s="17">
         <v>45716</v>
@@ -15292,19 +15292,19 @@
     </row>
     <row r="15" spans="1:8" ht="13">
       <c r="A15" s="58" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B15" s="24" t="s">
+        <v>214</v>
+      </c>
+      <c r="C15" s="61" t="s">
+        <v>215</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="E15" s="24" t="s">
         <v>216</v>
-      </c>
-      <c r="C15" s="61" t="s">
-        <v>217</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="E15" s="24" t="s">
-        <v>218</v>
       </c>
       <c r="F15" s="23">
         <v>45716</v>
@@ -15316,19 +15316,19 @@
     </row>
     <row r="16" spans="1:8" ht="42">
       <c r="A16" s="57" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B16" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>219</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>220</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>190</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>221</v>
       </c>
       <c r="F16" s="17">
         <v>45716</v>
@@ -15337,7 +15337,7 @@
         <v>45718</v>
       </c>
       <c r="H16" s="132" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="13">
@@ -18540,7 +18540,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="70" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C1" s="70" t="s">
         <v>6</v>
@@ -18566,16 +18566,16 @@
         <v>19</v>
       </c>
       <c r="B2" s="74" t="s">
+        <v>221</v>
+      </c>
+      <c r="C2" s="59" t="s">
+        <v>222</v>
+      </c>
+      <c r="D2" s="75" t="s">
+        <v>170</v>
+      </c>
+      <c r="E2" s="75" t="s">
         <v>223</v>
-      </c>
-      <c r="C2" s="59" t="s">
-        <v>224</v>
-      </c>
-      <c r="D2" s="75" t="s">
-        <v>172</v>
-      </c>
-      <c r="E2" s="75" t="s">
-        <v>225</v>
       </c>
       <c r="F2" s="76">
         <v>45716</v>
@@ -18587,19 +18587,19 @@
     </row>
     <row r="3" spans="1:8" ht="53">
       <c r="A3" s="78" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="21" t="s">
+        <v>224</v>
+      </c>
+      <c r="C3" s="126" t="s">
+        <v>405</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>225</v>
+      </c>
+      <c r="E3" s="24" t="s">
         <v>226</v>
-      </c>
-      <c r="C3" s="126" t="s">
-        <v>407</v>
-      </c>
-      <c r="D3" s="24" t="s">
-        <v>227</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>228</v>
       </c>
       <c r="F3" s="23">
         <v>45716</v>
@@ -18611,19 +18611,19 @@
     </row>
     <row r="4" spans="1:8" ht="53">
       <c r="A4" s="73" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F4" s="17">
         <v>45716</v>
@@ -18635,19 +18635,19 @@
     </row>
     <row r="5" spans="1:8" ht="40">
       <c r="A5" s="78" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C5" s="137" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F5" s="23">
         <v>45716</v>
@@ -18659,19 +18659,19 @@
     </row>
     <row r="6" spans="1:8" ht="14">
       <c r="A6" s="73" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>232</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>233</v>
       </c>
-      <c r="C6" s="59" t="s">
+      <c r="E6" s="18" t="s">
         <v>234</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>235</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>236</v>
       </c>
       <c r="F6" s="17">
         <v>45716</v>
@@ -18683,19 +18683,19 @@
     </row>
     <row r="7" spans="1:8" ht="40">
       <c r="A7" s="78" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="C7" s="81" t="s">
+        <v>236</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="E7" s="24" t="s">
         <v>237</v>
-      </c>
-      <c r="C7" s="81" t="s">
-        <v>238</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>239</v>
       </c>
       <c r="F7" s="23">
         <v>45716</v>
@@ -18707,19 +18707,19 @@
     </row>
     <row r="8" spans="1:8" ht="14">
       <c r="A8" s="73" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>239</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="E8" s="18" t="s">
         <v>240</v>
-      </c>
-      <c r="C8" s="59" t="s">
-        <v>241</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>242</v>
       </c>
       <c r="F8" s="17">
         <v>45716</v>
@@ -18731,19 +18731,19 @@
     </row>
     <row r="9" spans="1:8" ht="28">
       <c r="A9" s="78" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>242</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="E9" s="24" t="s">
         <v>243</v>
-      </c>
-      <c r="C9" s="59" t="s">
-        <v>244</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>245</v>
       </c>
       <c r="F9" s="23">
         <v>45716</v>
@@ -18755,19 +18755,19 @@
     </row>
     <row r="10" spans="1:8" ht="28">
       <c r="A10" s="73" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10" s="82" t="s">
+        <v>244</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>245</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="E10" s="18" t="s">
         <v>246</v>
-      </c>
-      <c r="C10" s="59" t="s">
-        <v>247</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>203</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>248</v>
       </c>
       <c r="F10" s="17">
         <v>45716</v>
@@ -18776,24 +18776,24 @@
         <v>45718</v>
       </c>
       <c r="H10" s="80" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="40">
       <c r="A11" s="78" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C11" s="138" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="F11" s="23">
         <v>45716</v>
@@ -18805,19 +18805,19 @@
     </row>
     <row r="12" spans="1:8" ht="28">
       <c r="A12" s="73" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>250</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" s="18" t="s">
         <v>251</v>
-      </c>
-      <c r="C12" s="59" t="s">
-        <v>252</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>211</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>253</v>
       </c>
       <c r="F12" s="17">
         <v>45716</v>
@@ -18829,19 +18829,19 @@
     </row>
     <row r="13" spans="1:8" ht="14">
       <c r="A13" s="78" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" s="21" t="s">
+        <v>252</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="E13" s="24" t="s">
         <v>254</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>255</v>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="E13" s="24" t="s">
-        <v>256</v>
       </c>
       <c r="F13" s="23">
         <v>45716</v>
@@ -18853,19 +18853,19 @@
     </row>
     <row r="14" spans="1:8" ht="28">
       <c r="A14" s="73" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="D14" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="E14" s="18" t="s">
         <v>258</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>259</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>260</v>
       </c>
       <c r="F14" s="17">
         <v>45716</v>
@@ -18877,19 +18877,19 @@
     </row>
     <row r="15" spans="1:8" ht="66">
       <c r="A15" s="78" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C15" s="126" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="F15" s="23">
         <v>45716</v>
@@ -18901,19 +18901,19 @@
     </row>
     <row r="16" spans="1:8" ht="14">
       <c r="A16" s="73" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>263</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>264</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>190</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>265</v>
       </c>
       <c r="F16" s="17">
         <v>45716</v>
@@ -22174,7 +22174,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="90" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C1" s="90" t="s">
         <v>6</v>
@@ -22200,16 +22200,16 @@
         <v>19</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="C2" s="33" t="s">
+        <v>265</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>266</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="E2" s="16" t="s">
         <v>267</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>269</v>
       </c>
       <c r="F2" s="43"/>
       <c r="G2" s="14"/>
@@ -22217,19 +22217,19 @@
     </row>
     <row r="3" spans="1:8" ht="56">
       <c r="A3" s="94" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>269</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="E3" s="22" t="s">
         <v>270</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>271</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>268</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>272</v>
       </c>
       <c r="F3" s="46"/>
       <c r="G3" s="21"/>
@@ -22237,19 +22237,19 @@
     </row>
     <row r="4" spans="1:8" ht="70">
       <c r="A4" s="92" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>272</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>266</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>273</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>274</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>275</v>
       </c>
       <c r="F4" s="43"/>
       <c r="G4" s="14"/>
@@ -22257,19 +22257,19 @@
     </row>
     <row r="5" spans="1:8" ht="42">
       <c r="A5" s="94" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" s="21" t="s">
+        <v>274</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>275</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="E5" s="21" t="s">
         <v>276</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>277</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>268</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>278</v>
       </c>
       <c r="F5" s="46"/>
       <c r="G5" s="21"/>
@@ -22277,19 +22277,19 @@
     </row>
     <row r="6" spans="1:8" ht="56">
       <c r="A6" s="92" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>266</v>
+      </c>
+      <c r="E6" s="16" t="s">
         <v>279</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>280</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>281</v>
       </c>
       <c r="F6" s="43"/>
       <c r="G6" s="14"/>
@@ -22297,19 +22297,19 @@
     </row>
     <row r="7" spans="1:8" ht="28">
       <c r="A7" s="94" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="21" t="s">
+        <v>280</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>410</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>281</v>
+      </c>
+      <c r="E7" s="22" t="s">
         <v>282</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>412</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>284</v>
       </c>
       <c r="F7" s="46"/>
       <c r="G7" s="21"/>
@@ -22317,19 +22317,19 @@
     </row>
     <row r="8" spans="1:8" ht="28">
       <c r="A8" s="92" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>284</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>285</v>
-      </c>
-      <c r="C8" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>283</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>287</v>
       </c>
       <c r="F8" s="43"/>
       <c r="G8" s="14"/>
@@ -22337,19 +22337,19 @@
     </row>
     <row r="9" spans="1:8" ht="28">
       <c r="A9" s="94" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="21" t="s">
+        <v>286</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>287</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>281</v>
+      </c>
+      <c r="E9" s="22" t="s">
         <v>288</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>289</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>290</v>
       </c>
       <c r="F9" s="46"/>
       <c r="G9" s="21"/>
@@ -22357,19 +22357,19 @@
     </row>
     <row r="10" spans="1:8" ht="14">
       <c r="A10" s="92" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>290</v>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="E10" s="14" t="s">
         <v>292</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>293</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>294</v>
       </c>
       <c r="F10" s="43"/>
       <c r="G10" s="14"/>
@@ -22377,19 +22377,19 @@
     </row>
     <row r="11" spans="1:8" ht="93">
       <c r="A11" s="94" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B11" s="21" t="s">
+        <v>293</v>
+      </c>
+      <c r="C11" s="126" t="s">
+        <v>411</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>294</v>
+      </c>
+      <c r="E11" s="21" t="s">
         <v>295</v>
-      </c>
-      <c r="C11" s="126" t="s">
-        <v>413</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>296</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>297</v>
       </c>
       <c r="F11" s="46"/>
       <c r="G11" s="21"/>
@@ -22397,19 +22397,19 @@
     </row>
     <row r="12" spans="1:8" ht="28">
       <c r="A12" s="92" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="E12" s="14" t="s">
         <v>298</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>299</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>293</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>300</v>
       </c>
       <c r="F12" s="43"/>
       <c r="G12" s="14"/>
@@ -22417,19 +22417,19 @@
     </row>
     <row r="13" spans="1:8" ht="28">
       <c r="A13" s="94" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>300</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>294</v>
+      </c>
+      <c r="E13" s="21" t="s">
         <v>301</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>302</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>296</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>303</v>
       </c>
       <c r="F13" s="46"/>
       <c r="G13" s="21"/>
@@ -30452,7 +30452,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="100" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C1" s="100" t="s">
         <v>6</v>
@@ -30478,16 +30478,16 @@
         <v>19</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="C2" s="104" t="s">
+        <v>303</v>
+      </c>
+      <c r="D2" s="83" t="s">
         <v>304</v>
       </c>
-      <c r="C2" s="104" t="s">
+      <c r="E2" s="16" t="s">
         <v>305</v>
-      </c>
-      <c r="D2" s="83" t="s">
-        <v>306</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>307</v>
       </c>
       <c r="F2" s="17">
         <v>45723</v>
@@ -30499,19 +30499,19 @@
     </row>
     <row r="3" spans="1:8" ht="42">
       <c r="A3" s="106" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>307</v>
+      </c>
+      <c r="D3" s="84" t="s">
+        <v>304</v>
+      </c>
+      <c r="E3" s="22" t="s">
         <v>308</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>309</v>
-      </c>
-      <c r="D3" s="84" t="s">
-        <v>306</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>310</v>
       </c>
       <c r="F3" s="23">
         <v>45723</v>
@@ -30523,19 +30523,19 @@
     </row>
     <row r="4" spans="1:8" ht="42">
       <c r="A4" s="103" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>309</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="D4" s="83" t="s">
+        <v>304</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>311</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>312</v>
-      </c>
-      <c r="D4" s="83" t="s">
-        <v>306</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>313</v>
       </c>
       <c r="F4" s="17">
         <v>45723</v>
@@ -30547,19 +30547,19 @@
     </row>
     <row r="5" spans="1:8" ht="42">
       <c r="A5" s="106" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" s="21" t="s">
+        <v>312</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>313</v>
+      </c>
+      <c r="D5" s="84" t="s">
         <v>314</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="E5" s="21" t="s">
         <v>315</v>
-      </c>
-      <c r="D5" s="84" t="s">
-        <v>316</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>317</v>
       </c>
       <c r="F5" s="23">
         <v>45723</v>
@@ -30571,19 +30571,19 @@
     </row>
     <row r="6" spans="1:8" ht="56">
       <c r="A6" s="103" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="D6" s="83" t="s">
         <v>318</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="E6" s="16" t="s">
         <v>319</v>
-      </c>
-      <c r="D6" s="83" t="s">
-        <v>320</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>321</v>
       </c>
       <c r="F6" s="17">
         <v>45723</v>
@@ -30595,19 +30595,19 @@
     </row>
     <row r="7" spans="1:8" ht="27">
       <c r="A7" s="106" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="21" t="s">
+        <v>320</v>
+      </c>
+      <c r="C7" s="108" t="s">
+        <v>321</v>
+      </c>
+      <c r="D7" s="84" t="s">
+        <v>304</v>
+      </c>
+      <c r="E7" s="22" t="s">
         <v>322</v>
-      </c>
-      <c r="C7" s="108" t="s">
-        <v>323</v>
-      </c>
-      <c r="D7" s="84" t="s">
-        <v>306</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>324</v>
       </c>
       <c r="F7" s="23">
         <v>45723</v>
@@ -30619,19 +30619,19 @@
     </row>
     <row r="8" spans="1:8" ht="28">
       <c r="A8" s="103" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>323</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>324</v>
+      </c>
+      <c r="D8" s="83" t="s">
+        <v>304</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>325</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>326</v>
-      </c>
-      <c r="D8" s="83" t="s">
-        <v>306</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>327</v>
       </c>
       <c r="F8" s="17">
         <v>45723</v>
@@ -30643,19 +30643,19 @@
     </row>
     <row r="9" spans="1:8" ht="14">
       <c r="A9" s="106" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="21" t="s">
+        <v>326</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>327</v>
+      </c>
+      <c r="D9" s="84" t="s">
+        <v>318</v>
+      </c>
+      <c r="E9" s="22" t="s">
         <v>328</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>329</v>
-      </c>
-      <c r="D9" s="84" t="s">
-        <v>320</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>330</v>
       </c>
       <c r="F9" s="23">
         <v>45723</v>
@@ -30667,19 +30667,19 @@
     </row>
     <row r="10" spans="1:8" ht="28">
       <c r="A10" s="103" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F10" s="17">
         <v>45723</v>
@@ -30691,19 +30691,19 @@
     </row>
     <row r="11" spans="1:8" ht="42">
       <c r="A11" s="106" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B11" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="D11" s="24" t="s">
         <v>333</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="E11" s="21" t="s">
         <v>334</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>335</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>336</v>
       </c>
       <c r="F11" s="23">
         <v>45723</v>
@@ -30715,19 +30715,19 @@
     </row>
     <row r="12" spans="1:8" ht="28">
       <c r="A12" s="103" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>335</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="D12" s="83" t="s">
+        <v>318</v>
+      </c>
+      <c r="E12" s="14" t="s">
         <v>337</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="D12" s="83" t="s">
-        <v>320</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>339</v>
       </c>
       <c r="F12" s="17">
         <v>45723</v>
@@ -30739,19 +30739,19 @@
     </row>
     <row r="13" spans="1:8" ht="56">
       <c r="A13" s="106" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B13" s="21" t="s">
+        <v>338</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="D13" s="84" t="s">
+        <v>314</v>
+      </c>
+      <c r="E13" s="21" t="s">
         <v>340</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>341</v>
-      </c>
-      <c r="D13" s="84" t="s">
-        <v>316</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>342</v>
       </c>
       <c r="F13" s="23">
         <v>45723</v>
@@ -30760,7 +30760,7 @@
         <v>45723</v>
       </c>
       <c r="H13" s="139" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="13">
@@ -34989,7 +34989,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="114" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C1" s="114" t="s">
         <v>6</v>
@@ -35015,16 +35015,16 @@
         <v>19</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>343</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="E2" s="16" t="s">
         <v>344</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>345</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>346</v>
       </c>
       <c r="F2" s="43">
         <v>45722</v>
@@ -35036,19 +35036,19 @@
     </row>
     <row r="3" spans="1:8" ht="26">
       <c r="A3" s="118" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="21" t="s">
+        <v>345</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>346</v>
+      </c>
+      <c r="D3" s="22" t="s">
         <v>347</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="E3" s="22" t="s">
         <v>348</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>349</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>350</v>
       </c>
       <c r="F3" s="46">
         <v>45722</v>
@@ -35060,19 +35060,19 @@
     </row>
     <row r="4" spans="1:8" ht="28">
       <c r="A4" s="116" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>349</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>350</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>347</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>351</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>352</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>349</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>353</v>
       </c>
       <c r="F4" s="43">
         <v>45722</v>
@@ -35084,19 +35084,19 @@
     </row>
     <row r="5" spans="1:8" ht="65">
       <c r="A5" s="118" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" s="21" t="s">
+        <v>352</v>
+      </c>
+      <c r="C5" s="126" t="s">
+        <v>414</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="E5" s="21" t="s">
         <v>354</v>
-      </c>
-      <c r="C5" s="126" t="s">
-        <v>416</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>355</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>356</v>
       </c>
       <c r="F5" s="46">
         <v>45722</v>
@@ -35108,19 +35108,19 @@
     </row>
     <row r="6" spans="1:8" ht="28">
       <c r="A6" s="116" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>355</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>356</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="E6" s="16" t="s">
         <v>357</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>358</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>355</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>359</v>
       </c>
       <c r="F6" s="43">
         <v>45722</v>
@@ -35132,19 +35132,19 @@
     </row>
     <row r="7" spans="1:8" ht="56">
       <c r="A7" s="118" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="21" t="s">
+        <v>358</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>359</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="E7" s="22" t="s">
         <v>360</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>361</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>355</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>362</v>
       </c>
       <c r="F7" s="46">
         <v>45722</v>
@@ -35156,19 +35156,19 @@
     </row>
     <row r="8" spans="1:8" ht="14">
       <c r="A8" s="116" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="C8" s="120" t="s">
+        <v>362</v>
+      </c>
+      <c r="D8" s="16" t="s">
         <v>363</v>
       </c>
-      <c r="C8" s="120" t="s">
+      <c r="E8" s="16" t="s">
         <v>364</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>365</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>366</v>
       </c>
       <c r="F8" s="43">
         <v>45722</v>
@@ -35180,19 +35180,19 @@
     </row>
     <row r="9" spans="1:8" ht="28">
       <c r="A9" s="118" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B9" s="21" t="s">
+        <v>365</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>366</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>343</v>
+      </c>
+      <c r="E9" s="21" t="s">
         <v>367</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>368</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>345</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>369</v>
       </c>
       <c r="F9" s="46">
         <v>45722</v>
@@ -35204,19 +35204,19 @@
     </row>
     <row r="10" spans="1:8" ht="28">
       <c r="A10" s="116" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>368</v>
+      </c>
+      <c r="C10" s="121" t="s">
+        <v>369</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>370</v>
-      </c>
-      <c r="C10" s="121" t="s">
-        <v>371</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>365</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>372</v>
       </c>
       <c r="F10" s="43">
         <v>45722</v>
@@ -35228,19 +35228,19 @@
     </row>
     <row r="11" spans="1:8" ht="28">
       <c r="A11" s="118" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B11" s="21" t="s">
+        <v>371</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>372</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>373</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="E11" s="21" t="s">
         <v>374</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>375</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>376</v>
       </c>
       <c r="F11" s="46">
         <v>45722</v>
@@ -35252,19 +35252,19 @@
     </row>
     <row r="12" spans="1:8" ht="319">
       <c r="A12" s="116" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>376</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E12" s="14" t="s">
         <v>377</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>379</v>
       </c>
       <c r="F12" s="43">
         <v>45722</v>
@@ -35276,19 +35276,19 @@
     </row>
     <row r="13" spans="1:8" ht="28">
       <c r="A13" s="118" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B13" s="24" t="s">
+        <v>378</v>
+      </c>
+      <c r="C13" s="122" t="s">
+        <v>379</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="E13" s="21" t="s">
         <v>380</v>
-      </c>
-      <c r="C13" s="122" t="s">
-        <v>381</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>382</v>
       </c>
       <c r="F13" s="46">
         <v>45722</v>
@@ -35300,19 +35300,19 @@
     </row>
     <row r="14" spans="1:8" ht="42">
       <c r="A14" s="116" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B14" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>382</v>
+      </c>
+      <c r="D14" s="14" t="s">
         <v>383</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="E14" s="14" t="s">
         <v>384</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>385</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>386</v>
       </c>
       <c r="F14" s="43">
         <v>45722</v>
@@ -35324,19 +35324,19 @@
     </row>
     <row r="15" spans="1:8" ht="14">
       <c r="A15" s="118" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B15" s="24" t="s">
+        <v>385</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>386</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>383</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>387</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>388</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>385</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>389</v>
       </c>
       <c r="F15" s="46">
         <v>45722</v>
@@ -35348,19 +35348,19 @@
     </row>
     <row r="16" spans="1:8" ht="14">
       <c r="A16" s="116" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B16" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>389</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="E16" s="14" t="s">
         <v>390</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>391</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>385</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>392</v>
       </c>
       <c r="F16" s="43">
         <v>45722</v>
@@ -35372,19 +35372,19 @@
     </row>
     <row r="17" spans="1:8" ht="84">
       <c r="A17" s="116" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B17" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="D17" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>394</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="13">

</xml_diff>

<commit_message>
update new chat text black, fix issue with query finding results on vector store
</commit_message>
<xml_diff>
--- a/uploaded_files/EMERGE Content - Capstone ITSMF.xlsx
+++ b/uploaded_files/EMERGE Content - Capstone ITSMF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aieshadotson/Code_Repos/ITSMF_Chatbot/chatbot-prototype/uploaded_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC512398-5FD4-8042-8A97-21332BDE1915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CFD080-8758-D247-BCB7-6E52D57089AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1040" windowWidth="60160" windowHeight="28240" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legend" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="439">
   <si>
     <t>Title</t>
   </si>
@@ -1113,6 +1113,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>. You will need to fill out your contact information.</t>
@@ -1164,6 +1165,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>, so it’s easy to find one that matches your skills, interests, and availability.</t>
@@ -1212,6 +1214,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>. You will need to fill out your contact information.</t>
@@ -1251,6 +1254,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">. </t>
@@ -1302,6 +1306,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">. </t>
@@ -1332,6 +1337,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
@@ -1407,6 +1413,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
@@ -1503,6 +1510,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> to stay connected. </t>
@@ -1536,6 +1544,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">, </t>
@@ -1555,6 +1564,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">, </t>
@@ -1574,6 +1584,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">, and </t>
@@ -1684,6 +1695,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> where candidates and employers can find careers and search for diverse talent. </t>
@@ -1696,9 +1708,6 @@
     <t xml:space="preserve">Who is the President and CEO of ITSMF? </t>
   </si>
   <si>
-    <t>Johanna R. Jones</t>
-  </si>
-  <si>
     <t>Leadership &amp; Governance</t>
   </si>
   <si>
@@ -1763,12 +1772,6 @@
   <si>
     <t xml:space="preserve">ITSMF has partnered with MindEdge to provide exclusive online professional development courses. With over 300 self-paced courses across 30+ categories, members can learn anytime, anywhere—plus enjoy a 10% discount using code ITSMF10 at checkout.
 </t>
-  </si>
-  <si>
-    <t>Professional Development &amp; Education</t>
-  </si>
-  <si>
-    <t>learning, courses, training, development, education, certification, professional growth, online classes, skills improvement</t>
   </si>
   <si>
     <t>Business leaders who embody visionary leadership, a global mindset and a passion for family, community and social activism may qualify for ITSMF Executive Membership. Prospective members must work at the director-level and above, be sponsored by an existing ITSMF member and complete an application to ensure their genuine commitment to increasing dynamic leadership by supporting current and future technology leaders.</t>
@@ -2082,12 +2085,87 @@
   <si>
     <t>Management Academy, Mid-Level professional, men, women</t>
   </si>
+  <si>
+    <t>What are members saying about the impact of ITSMF?</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Dh18-rZjzBdIEHCh6fyZA76x-OVN7m0j/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is ITSMF history? </t>
+  </si>
+  <si>
+    <t>What are partners saying about the impact of ITSMF?</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1wMRmzxdo7nB9vIbooFq6x7lVwU2CGDd5/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>Q29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What are academy members saying? </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1AY5ctKpPpntxqgouHa01NR_Oxm_Akaz7/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>Q30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What are EMERGE Academy members saying? </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1xGWYMuf81O5-O_X2enf4egTTApHsd7Gt/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>Academies, feedback, impact, benefits, testimonial video</t>
+  </si>
+  <si>
+    <t>EMERGE, feedback, impact, benefits, testimonial video</t>
+  </si>
+  <si>
+    <t>Membership &amp; Engagement</t>
+  </si>
+  <si>
+    <t>testimonials, feedback, impact, success stories</t>
+  </si>
+  <si>
+    <t>Organizational Background &amp; Identity</t>
+  </si>
+  <si>
+    <t>story, background, founding, origins</t>
+  </si>
+  <si>
+    <t>What is ITSMF?</t>
+  </si>
+  <si>
+    <t>ITSMF is a professional and personal leadership development program for people of color.  Their mission is to increase the representation of professionals at senior levels in technology, to impact organizational innovation and growth by developing and nurturing dynamic leaders through enrichment of the mind, body, and soul. You can find more information at: https://itsmfleaders.org/about-itsmf/.</t>
+  </si>
+  <si>
+    <t>ITSMF, about, overview, organization</t>
+  </si>
+  <si>
+    <t>Testimonials</t>
+  </si>
+  <si>
+    <t>external partner testimonial, sponsor testimonial, feedback, impact, experiences</t>
+  </si>
+  <si>
+    <t>testimonials, feedback, impact, success stories, history</t>
+  </si>
+  <si>
+    <t>Here about ITSMF History Here  https://drive.google.com/file/d/18c425MS617SaGuRQyFEuueBOij4jbrc0/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>The current President and CEO of the Information Technology Senior Management Forum (ITSMF) is Johanna R. Jones. She was appointed in August 2021, succeeding retiring executive Viola Maxwell-Thompson. Johanna brings over 20 years of nonprofit executive leadership experience, with deep expertise in fundraising, strategic partnerships, and workforce development. Prior to joining ITSMF, she served as Director of Workforce Development and Strategic Partnerships at Southern Illinois University Edwardsville and as Vice President of Development and Advancement at Places for People, where she successfully led a $7 million capital campaign. She holds a Bachelor of Science in Mass Communications from Jackson State University and a Juris Doctorate from St. Louis University School of Law. Johanna is also active in several charitable organizations and nonprofit boards, including Jack and Jill of America and Delta Sigma Theta Sorority, Inc. You can reach her directly at president@itsmfleaders.org.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2255,6 +2333,14 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -3588,10 +3674,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4010,8 +4097,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="25">
@@ -4371,7 +4474,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="General_Info" displayName="General_Info" ref="A1:H50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="General_Info" displayName="General_Info" ref="A1:H53">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Question ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="User Question"/>
@@ -4755,7 +4858,7 @@
         <v>22</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="F2" s="17">
         <v>45718</v>
@@ -4777,7 +4880,7 @@
         <v>22</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="F3" s="23">
         <v>45718</v>
@@ -5355,23 +5458,47 @@
       <c r="G29" s="24"/>
       <c r="H29" s="25"/>
     </row>
-    <row r="30" spans="1:8" ht="13">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="18"/>
+    <row r="30" spans="1:8" ht="28">
+      <c r="A30" s="13" t="s">
+        <v>419</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>420</v>
+      </c>
+      <c r="C30" s="142" t="s">
+        <v>421</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>425</v>
+      </c>
+      <c r="F30" s="23">
+        <v>45718</v>
+      </c>
       <c r="G30" s="18"/>
       <c r="H30" s="19"/>
     </row>
-    <row r="31" spans="1:8" ht="13">
-      <c r="A31" s="20"/>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="24"/>
+    <row r="31" spans="1:8" ht="28">
+      <c r="A31" s="20" t="s">
+        <v>422</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>423</v>
+      </c>
+      <c r="C31" s="144" t="s">
+        <v>424</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" s="21" t="s">
+        <v>426</v>
+      </c>
+      <c r="F31" s="23">
+        <v>45718</v>
+      </c>
       <c r="G31" s="24"/>
       <c r="H31" s="25"/>
     </row>
@@ -5592,10 +5719,12 @@
     <hyperlink ref="C27" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
     <hyperlink ref="C28" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
     <hyperlink ref="C29" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="C30" r:id="rId4" xr:uid="{D7582636-E9A9-7046-BF35-083DBC3640A2}"/>
+    <hyperlink ref="C31" r:id="rId5" xr:uid="{561CE403-B50A-A246-898F-BFBB174DE448}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5675,7 +5804,7 @@
         <v>127</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="D3" s="21" t="s">
         <v>125</v>
@@ -5891,7 +6020,7 @@
         <v>152</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>125</v>
@@ -5963,7 +6092,7 @@
         <v>157</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>125</v>
@@ -14991,7 +15120,7 @@
         <v>45718</v>
       </c>
       <c r="H2" s="129" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="117">
@@ -15002,7 +15131,7 @@
         <v>172</v>
       </c>
       <c r="C3" s="126" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="D3" s="24" t="s">
         <v>173</v>
@@ -15124,7 +15253,7 @@
         <v>190</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="D8" s="18" t="s">
         <v>173</v>
@@ -15150,7 +15279,7 @@
         <v>192</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="D9" s="24" t="s">
         <v>193</v>
@@ -15248,7 +15377,7 @@
         <v>208</v>
       </c>
       <c r="C13" s="127" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="D13" s="24" t="s">
         <v>209</v>
@@ -15263,7 +15392,7 @@
         <v>45718</v>
       </c>
       <c r="H13" s="130" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="13">
@@ -15337,7 +15466,7 @@
         <v>45718</v>
       </c>
       <c r="H16" s="132" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="13">
@@ -18593,7 +18722,7 @@
         <v>224</v>
       </c>
       <c r="C3" s="126" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="D3" s="24" t="s">
         <v>225</v>
@@ -18617,7 +18746,7 @@
         <v>227</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="D4" s="18" t="s">
         <v>225</v>
@@ -18641,7 +18770,7 @@
         <v>229</v>
       </c>
       <c r="C5" s="137" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D5" s="24" t="s">
         <v>225</v>
@@ -18787,7 +18916,7 @@
         <v>247</v>
       </c>
       <c r="C11" s="138" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="D11" s="24" t="s">
         <v>206</v>
@@ -18883,7 +19012,7 @@
         <v>259</v>
       </c>
       <c r="C15" s="126" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="D15" s="24" t="s">
         <v>257</v>
@@ -18923,12 +19052,22 @@
       </c>
       <c r="H16" s="80"/>
     </row>
-    <row r="17" spans="1:8" ht="13">
-      <c r="A17" s="73"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
+    <row r="17" spans="1:8" ht="28">
+      <c r="A17" s="73" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>417</v>
+      </c>
+      <c r="C17" s="143" t="s">
+        <v>418</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>434</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>435</v>
+      </c>
       <c r="F17" s="17"/>
       <c r="G17" s="18"/>
       <c r="H17" s="80"/>
@@ -22143,10 +22282,11 @@
     <hyperlink ref="C11" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
     <hyperlink ref="C12" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
     <hyperlink ref="C15" r:id="rId12" location="donate" display="Our payment options for making a donation are PayPal or Credit Card.  Payments can be made at the following site by clicking the Donate button._x000a_https://itsmfleaders.org/engage/#donate" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
+    <hyperlink ref="C17" r:id="rId13" xr:uid="{FF4EF1B0-5DF0-A949-B85F-E7F2FA834A2A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
@@ -22303,7 +22443,7 @@
         <v>280</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>281</v>
@@ -22383,7 +22523,7 @@
         <v>293</v>
       </c>
       <c r="C11" s="126" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>294</v>
@@ -30673,7 +30813,7 @@
         <v>329</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D10" s="18" t="s">
         <v>318</v>
@@ -30760,7 +30900,7 @@
         <v>45723</v>
       </c>
       <c r="H13" s="139" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="13">
@@ -34971,7 +35111,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H996"/>
+  <dimension ref="A1:H999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -35090,7 +35230,7 @@
         <v>352</v>
       </c>
       <c r="C5" s="126" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>353</v>
@@ -35226,7 +35366,7 @@
       </c>
       <c r="H10" s="117"/>
     </row>
-    <row r="11" spans="1:8" ht="28">
+    <row r="11" spans="1:8" ht="238">
       <c r="A11" s="118" t="s">
         <v>58</v>
       </c>
@@ -35234,13 +35374,13 @@
         <v>371</v>
       </c>
       <c r="C11" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>372</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="E11" s="21" t="s">
         <v>373</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>374</v>
       </c>
       <c r="F11" s="46">
         <v>45722</v>
@@ -35255,16 +35395,16 @@
         <v>62</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>374</v>
+      </c>
+      <c r="C12" s="14" t="s">
         <v>375</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>376</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>125</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F12" s="43">
         <v>45722</v>
@@ -35279,16 +35419,16 @@
         <v>65</v>
       </c>
       <c r="B13" s="24" t="s">
+        <v>377</v>
+      </c>
+      <c r="C13" s="122" t="s">
         <v>378</v>
-      </c>
-      <c r="C13" s="122" t="s">
-        <v>379</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>125</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F13" s="46">
         <v>45722</v>
@@ -35303,16 +35443,16 @@
         <v>69</v>
       </c>
       <c r="B14" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>381</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" s="14" t="s">
         <v>382</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="E14" s="14" t="s">
         <v>383</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>384</v>
       </c>
       <c r="F14" s="43">
         <v>45722</v>
@@ -35327,16 +35467,16 @@
         <v>73</v>
       </c>
       <c r="B15" s="24" t="s">
+        <v>384</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>385</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="D15" s="21" t="s">
+        <v>382</v>
+      </c>
+      <c r="E15" s="21" t="s">
         <v>386</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>383</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>387</v>
       </c>
       <c r="F15" s="46">
         <v>45722</v>
@@ -35351,16 +35491,16 @@
         <v>77</v>
       </c>
       <c r="B16" s="18" t="s">
+        <v>387</v>
+      </c>
+      <c r="C16" s="14" t="s">
         <v>388</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="D16" s="14" t="s">
+        <v>382</v>
+      </c>
+      <c r="E16" s="14" t="s">
         <v>389</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>383</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>390</v>
       </c>
       <c r="F16" s="43">
         <v>45722</v>
@@ -35370,369 +35510,417 @@
       </c>
       <c r="H16" s="117"/>
     </row>
-    <row r="17" spans="1:8" ht="84">
+    <row r="17" spans="1:8" ht="28">
       <c r="A17" s="116" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>414</v>
+      </c>
+      <c r="C17" s="142" t="s">
+        <v>415</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>428</v>
+      </c>
+      <c r="F17" s="43">
+        <v>45722</v>
+      </c>
+      <c r="G17" s="43">
+        <v>45722</v>
+      </c>
+      <c r="H17" s="141"/>
+    </row>
+    <row r="18" spans="1:8" ht="42">
+      <c r="A18" s="116" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="C18" s="142" t="s">
+        <v>437</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>427</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>436</v>
+      </c>
+      <c r="F18" s="43">
+        <v>45722</v>
+      </c>
+      <c r="G18" s="43">
+        <v>45722</v>
+      </c>
+      <c r="H18" s="141"/>
+    </row>
+    <row r="19" spans="1:8" ht="98">
+      <c r="A19" s="116" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="C19" s="142" t="s">
+        <v>432</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>429</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>433</v>
+      </c>
+      <c r="F19" s="140">
+        <v>45718</v>
+      </c>
+      <c r="G19" s="140">
+        <v>45718</v>
+      </c>
+      <c r="H19" s="141"/>
+    </row>
+    <row r="20" spans="1:8" ht="84">
+      <c r="A20" s="116" t="s">
         <v>93</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B20" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>391</v>
       </c>
-      <c r="C17" s="14" t="s">
-        <v>392</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="13">
-      <c r="A18" s="118"/>
-    </row>
-    <row r="19" spans="1:8" ht="13">
-      <c r="A19" s="116"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="43"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="117"/>
-    </row>
-    <row r="20" spans="1:8" ht="13">
-      <c r="A20" s="118"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="119"/>
+      <c r="D20" s="14" t="s">
+        <v>429</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="13">
-      <c r="A21" s="116"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="117"/>
+      <c r="A21" s="118"/>
     </row>
     <row r="22" spans="1:8" ht="13">
-      <c r="A22" s="118"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="119"/>
+      <c r="A22" s="116"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="117"/>
     </row>
     <row r="23" spans="1:8" ht="13">
-      <c r="A23" s="116"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="117"/>
+      <c r="A23" s="118"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="119"/>
     </row>
     <row r="24" spans="1:8" ht="13">
-      <c r="A24" s="118"/>
-      <c r="B24" s="21"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="119"/>
+      <c r="A24" s="116"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="117"/>
     </row>
     <row r="25" spans="1:8" ht="13">
-      <c r="A25" s="116"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="117"/>
+      <c r="A25" s="118"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="119"/>
     </row>
     <row r="26" spans="1:8" ht="13">
-      <c r="A26" s="118"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="119"/>
+      <c r="A26" s="116"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="117"/>
     </row>
     <row r="27" spans="1:8" ht="13">
-      <c r="A27" s="116"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="117"/>
+      <c r="A27" s="118"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="119"/>
     </row>
     <row r="28" spans="1:8" ht="13">
-      <c r="A28" s="118"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="119"/>
+      <c r="A28" s="116"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="117"/>
     </row>
     <row r="29" spans="1:8" ht="13">
-      <c r="A29" s="116"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="117"/>
+      <c r="A29" s="118"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="119"/>
     </row>
     <row r="30" spans="1:8" ht="13">
-      <c r="A30" s="118"/>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="119"/>
+      <c r="A30" s="116"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="117"/>
     </row>
     <row r="31" spans="1:8" ht="13">
-      <c r="A31" s="116"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="117"/>
+      <c r="A31" s="118"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="119"/>
     </row>
     <row r="32" spans="1:8" ht="13">
-      <c r="A32" s="118"/>
-      <c r="B32" s="21"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="119"/>
+      <c r="A32" s="116"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="117"/>
     </row>
     <row r="33" spans="1:8" ht="13">
-      <c r="A33" s="116"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="117"/>
+      <c r="A33" s="118"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="119"/>
     </row>
     <row r="34" spans="1:8" ht="13">
-      <c r="A34" s="118"/>
-      <c r="B34" s="21"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="119"/>
+      <c r="A34" s="116"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="117"/>
     </row>
     <row r="35" spans="1:8" ht="13">
-      <c r="A35" s="116"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="117"/>
+      <c r="A35" s="118"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="119"/>
     </row>
     <row r="36" spans="1:8" ht="13">
-      <c r="A36" s="118"/>
-      <c r="B36" s="21"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="119"/>
+      <c r="A36" s="116"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="117"/>
     </row>
     <row r="37" spans="1:8" ht="13">
-      <c r="A37" s="116"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="117"/>
+      <c r="A37" s="118"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="22"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="21"/>
+      <c r="H37" s="119"/>
     </row>
     <row r="38" spans="1:8" ht="13">
-      <c r="A38" s="118"/>
-      <c r="B38" s="21"/>
-      <c r="C38" s="22"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
-      <c r="G38" s="21"/>
-      <c r="H38" s="119"/>
+      <c r="A38" s="116"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="117"/>
     </row>
     <row r="39" spans="1:8" ht="13">
-      <c r="A39" s="116"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="117"/>
+      <c r="A39" s="118"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="119"/>
     </row>
     <row r="40" spans="1:8" ht="13">
-      <c r="A40" s="118"/>
-      <c r="B40" s="21"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
-      <c r="H40" s="119"/>
+      <c r="A40" s="116"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="117"/>
     </row>
     <row r="41" spans="1:8" ht="13">
-      <c r="A41" s="116"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="117"/>
+      <c r="A41" s="118"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="119"/>
     </row>
     <row r="42" spans="1:8" ht="13">
-      <c r="A42" s="118"/>
-      <c r="B42" s="21"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21"/>
-      <c r="G42" s="21"/>
-      <c r="H42" s="119"/>
+      <c r="A42" s="116"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="117"/>
     </row>
     <row r="43" spans="1:8" ht="13">
-      <c r="A43" s="116"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="117"/>
+      <c r="A43" s="118"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="21"/>
+      <c r="H43" s="119"/>
     </row>
     <row r="44" spans="1:8" ht="13">
-      <c r="A44" s="118"/>
-      <c r="B44" s="21"/>
-      <c r="C44" s="22"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="21"/>
-      <c r="F44" s="21"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="119"/>
+      <c r="A44" s="116"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="117"/>
     </row>
     <row r="45" spans="1:8" ht="13">
-      <c r="A45" s="116"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="117"/>
+      <c r="A45" s="118"/>
+      <c r="B45" s="21"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
+      <c r="H45" s="119"/>
     </row>
     <row r="46" spans="1:8" ht="13">
-      <c r="A46" s="118"/>
-      <c r="B46" s="21"/>
-      <c r="C46" s="22"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
-      <c r="H46" s="119"/>
+      <c r="A46" s="116"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
+      <c r="H46" s="117"/>
     </row>
     <row r="47" spans="1:8" ht="13">
-      <c r="A47" s="116"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="117"/>
+      <c r="A47" s="118"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="21"/>
+      <c r="H47" s="119"/>
     </row>
     <row r="48" spans="1:8" ht="13">
-      <c r="A48" s="118"/>
-      <c r="B48" s="21"/>
-      <c r="C48" s="22"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
-      <c r="H48" s="119"/>
+      <c r="A48" s="116"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="14"/>
+      <c r="G48" s="14"/>
+      <c r="H48" s="117"/>
     </row>
     <row r="49" spans="1:8" ht="13">
-      <c r="A49" s="116"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="16"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="117"/>
+      <c r="A49" s="118"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="21"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="21"/>
+      <c r="H49" s="119"/>
     </row>
     <row r="50" spans="1:8" ht="13">
-      <c r="A50" s="123"/>
-      <c r="B50" s="124"/>
-      <c r="C50" s="124"/>
-      <c r="D50" s="124"/>
-      <c r="E50" s="124"/>
-      <c r="F50" s="124"/>
-      <c r="G50" s="124"/>
-      <c r="H50" s="125"/>
+      <c r="A50" s="116"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="14"/>
+      <c r="E50" s="14"/>
+      <c r="F50" s="14"/>
+      <c r="G50" s="14"/>
+      <c r="H50" s="117"/>
     </row>
     <row r="51" spans="1:8" ht="13">
-      <c r="C51" s="53"/>
-      <c r="D51" s="53"/>
-      <c r="E51" s="53"/>
-      <c r="F51" s="53"/>
-      <c r="G51" s="53"/>
-      <c r="H51" s="53"/>
+      <c r="A51" s="118"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="21"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="21"/>
+      <c r="G51" s="21"/>
+      <c r="H51" s="119"/>
     </row>
     <row r="52" spans="1:8" ht="13">
-      <c r="C52" s="53"/>
-      <c r="D52" s="53"/>
-      <c r="E52" s="53"/>
-      <c r="F52" s="53"/>
-      <c r="G52" s="53"/>
-      <c r="H52" s="53"/>
+      <c r="A52" s="116"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="16"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="117"/>
     </row>
     <row r="53" spans="1:8" ht="13">
-      <c r="C53" s="53"/>
-      <c r="D53" s="53"/>
-      <c r="E53" s="53"/>
-      <c r="F53" s="53"/>
-      <c r="G53" s="53"/>
-      <c r="H53" s="53"/>
+      <c r="A53" s="123"/>
+      <c r="B53" s="124"/>
+      <c r="C53" s="124"/>
+      <c r="D53" s="124"/>
+      <c r="E53" s="124"/>
+      <c r="F53" s="124"/>
+      <c r="G53" s="124"/>
+      <c r="H53" s="125"/>
     </row>
     <row r="54" spans="1:8" ht="13">
       <c r="C54" s="53"/>
@@ -43277,6 +43465,30 @@
       <c r="F996" s="53"/>
       <c r="G996" s="53"/>
       <c r="H996" s="53"/>
+    </row>
+    <row r="997" spans="3:8" ht="13">
+      <c r="C997" s="53"/>
+      <c r="D997" s="53"/>
+      <c r="E997" s="53"/>
+      <c r="F997" s="53"/>
+      <c r="G997" s="53"/>
+      <c r="H997" s="53"/>
+    </row>
+    <row r="998" spans="3:8" ht="13">
+      <c r="C998" s="53"/>
+      <c r="D998" s="53"/>
+      <c r="E998" s="53"/>
+      <c r="F998" s="53"/>
+      <c r="G998" s="53"/>
+      <c r="H998" s="53"/>
+    </row>
+    <row r="999" spans="3:8" ht="13">
+      <c r="C999" s="53"/>
+      <c r="D999" s="53"/>
+      <c r="E999" s="53"/>
+      <c r="F999" s="53"/>
+      <c r="G999" s="53"/>
+      <c r="H999" s="53"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -43286,10 +43498,12 @@
     <hyperlink ref="C8" r:id="rId4" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
     <hyperlink ref="C10" r:id="rId5" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
     <hyperlink ref="C13" r:id="rId6" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
+    <hyperlink ref="C17" r:id="rId7" xr:uid="{A4CEEA82-842B-284D-8BF8-CD61B733DAC3}"/>
+    <hyperlink ref="C18" r:id="rId8" display="https://drive.google.com/file/d/18c425MS617SaGuRQyFEuueBOij4jbrc0/view?usp=drive_link" xr:uid="{B3D2D1FC-756A-634F-AA0B-43EC91A7B732}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>